<commit_message>
feat: map product holding cost percentages from Excel and update UI solver
</commit_message>
<xml_diff>
--- a/frontend/src/data/Product Master Ptototype.xlsx
+++ b/frontend/src/data/Product Master Ptototype.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SOMESH_\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3AF7905-0955-4F4E-B25B-1688B30AD4A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D1E95A0-2031-4BF5-8DD4-A72E761AF34B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A8F744CE-2ACC-42A0-AFFE-E37E74C81C0F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="92">
   <si>
     <t>ERP Code</t>
   </si>
@@ -62,9 +62,6 @@
     <t>Electrical</t>
   </si>
   <si>
-    <t>Discreption</t>
-  </si>
-  <si>
     <t>PRD0001</t>
   </si>
   <si>
@@ -294,6 +291,27 @@
   </si>
   <si>
     <t>In-Transit Inventory (Nos)</t>
+  </si>
+  <si>
+    <t>Cost/Unit $</t>
+  </si>
+  <si>
+    <t>ROP (Nos)</t>
+  </si>
+  <si>
+    <t>Daily Use (Nos)</t>
+  </si>
+  <si>
+    <t>Wt. Avg Lead Time (Days)</t>
+  </si>
+  <si>
+    <t>Holding cost - % of unit cost /unit/day</t>
+  </si>
+  <si>
+    <t>Holding Cost/Unit/Day</t>
+  </si>
+  <si>
+    <t>Discription</t>
   </si>
 </sst>
 </file>
@@ -303,7 +321,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-1009]#,##0.00"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -325,6 +343,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -340,7 +365,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -361,18 +386,33 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
@@ -706,7 +746,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29CFC8CC-25F2-4C56-B2E2-78563C8A1E95}">
-  <dimension ref="A1:K31"/>
+  <dimension ref="A1:Q31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.5546875" customWidth="1"/>
@@ -714,13 +754,19 @@
     <col min="3" max="4" width="20" customWidth="1"/>
     <col min="5" max="5" width="15.77734375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="20" customWidth="1"/>
-    <col min="10" max="10" width="13.109375" customWidth="1"/>
-    <col min="11" max="11" width="20" customWidth="1"/>
+    <col min="7" max="7" width="14.109375" customWidth="1"/>
+    <col min="8" max="8" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="20" customWidth="1"/>
+    <col min="11" max="11" width="13.109375" customWidth="1"/>
+    <col min="12" max="12" width="20" customWidth="1"/>
+    <col min="13" max="13" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.33203125" customWidth="1"/>
+    <col min="16" max="16" width="28.77734375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="26.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -731,42 +777,60 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>8</v>
+        <v>91</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>85</v>
       </c>
       <c r="H1" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="J1" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="I1" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="K1" s="2" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+      <c r="L1" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="N1" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="O1" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="P1" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="Q1" s="4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" ht="15" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B2">
         <v>870899</v>
       </c>
       <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
         <v>10</v>
-      </c>
-      <c r="D2" t="s">
-        <v>11</v>
       </c>
       <c r="E2">
         <v>12</v>
@@ -774,34 +838,56 @@
       <c r="F2" s="3">
         <v>144000</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="3">
+        <f>F2/E2</f>
+        <v>12000</v>
+      </c>
+      <c r="H2">
         <v>6</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>45</v>
       </c>
-      <c r="I2">
+      <c r="J2">
         <v>4</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>5</v>
       </c>
-      <c r="K2">
+      <c r="L2">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+      <c r="M2" s="5">
+        <v>24</v>
+      </c>
+      <c r="N2" s="6">
+        <f>E2/I2</f>
+        <v>0.26666666666666666</v>
+      </c>
+      <c r="O2" s="5">
+        <f>(N2*M2)+L2</f>
+        <v>9.4</v>
+      </c>
+      <c r="P2" s="7">
+        <v>8.0000000000000004E-4</v>
+      </c>
+      <c r="Q2" s="3">
+        <f>P2*G2</f>
+        <v>9.6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" ht="15" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B3">
         <v>840999</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E3">
         <v>120</v>
@@ -809,34 +895,56 @@
       <c r="F3" s="3">
         <v>3600</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="3">
+        <f t="shared" ref="G3:G31" si="0">F3/E3</f>
+        <v>30</v>
+      </c>
+      <c r="H3">
         <v>40</v>
       </c>
-      <c r="H3">
+      <c r="I3">
         <v>60</v>
       </c>
-      <c r="I3">
+      <c r="J3">
         <v>50</v>
       </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
         <v>5</v>
       </c>
-      <c r="K3">
+      <c r="L3">
         <v>20</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+      <c r="M3" s="5">
+        <v>15.5</v>
+      </c>
+      <c r="N3" s="6">
+        <f t="shared" ref="N3:N31" si="1">E3/I3</f>
+        <v>2</v>
+      </c>
+      <c r="O3" s="5">
+        <f t="shared" ref="O3:O31" si="2">(N3*M3)+L3</f>
+        <v>51</v>
+      </c>
+      <c r="P3" s="7">
+        <v>1.1000000000000001E-3</v>
+      </c>
+      <c r="Q3" s="3">
+        <f t="shared" ref="Q3:Q31" si="3">P3*G3</f>
+        <v>3.3000000000000002E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" ht="15" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B4">
         <v>870880</v>
       </c>
       <c r="C4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" t="s">
         <v>15</v>
-      </c>
-      <c r="D4" t="s">
-        <v>16</v>
       </c>
       <c r="E4">
         <v>45</v>
@@ -844,34 +952,56 @@
       <c r="F4" s="3">
         <v>13500</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="3">
+        <f t="shared" si="0"/>
+        <v>300</v>
+      </c>
+      <c r="H4">
         <v>10</v>
       </c>
-      <c r="H4">
+      <c r="I4">
         <v>30</v>
       </c>
-      <c r="I4">
+      <c r="J4">
         <v>10</v>
       </c>
-      <c r="J4" t="s">
+      <c r="K4" t="s">
         <v>5</v>
       </c>
-      <c r="K4">
+      <c r="L4">
         <v>5</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+      <c r="M4" s="5">
+        <v>26.5</v>
+      </c>
+      <c r="N4" s="6">
+        <f t="shared" si="1"/>
+        <v>1.5</v>
+      </c>
+      <c r="O4" s="5">
+        <f t="shared" si="2"/>
+        <v>44.75</v>
+      </c>
+      <c r="P4" s="7">
+        <v>5.9999999999999995E-4</v>
+      </c>
+      <c r="Q4" s="3">
+        <f t="shared" si="3"/>
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" ht="15" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B5">
         <v>870830</v>
       </c>
       <c r="C5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" t="s">
         <v>18</v>
-      </c>
-      <c r="D5" t="s">
-        <v>19</v>
       </c>
       <c r="E5">
         <v>8</v>
@@ -879,34 +1009,56 @@
       <c r="F5" s="3">
         <v>48000</v>
       </c>
-      <c r="G5">
+      <c r="G5" s="3">
+        <f t="shared" si="0"/>
+        <v>6000</v>
+      </c>
+      <c r="H5">
         <v>2</v>
       </c>
-      <c r="H5">
+      <c r="I5">
         <v>25</v>
       </c>
-      <c r="I5">
+      <c r="J5">
         <v>2</v>
       </c>
-      <c r="J5" t="s">
+      <c r="K5" t="s">
         <v>5</v>
       </c>
-      <c r="K5">
+      <c r="L5">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+      <c r="M5" s="5">
+        <v>36.4</v>
+      </c>
+      <c r="N5" s="6">
+        <f t="shared" si="1"/>
+        <v>0.32</v>
+      </c>
+      <c r="O5" s="5">
+        <f t="shared" si="2"/>
+        <v>12.648</v>
+      </c>
+      <c r="P5" s="7">
+        <v>1.4E-3</v>
+      </c>
+      <c r="Q5" s="3">
+        <f t="shared" si="3"/>
+        <v>8.4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" ht="15" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B6">
         <v>870840</v>
       </c>
       <c r="C6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E6">
         <v>6</v>
@@ -914,34 +1066,56 @@
       <c r="F6" s="3">
         <v>72000</v>
       </c>
-      <c r="G6">
+      <c r="G6" s="3">
+        <f t="shared" si="0"/>
+        <v>12000</v>
+      </c>
+      <c r="H6">
         <v>1</v>
       </c>
-      <c r="H6">
+      <c r="I6">
         <v>20</v>
       </c>
-      <c r="I6">
+      <c r="J6">
         <v>1</v>
       </c>
-      <c r="J6" t="s">
+      <c r="K6" t="s">
         <v>5</v>
       </c>
-      <c r="K6">
+      <c r="L6">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+      <c r="M6" s="5">
+        <v>36</v>
+      </c>
+      <c r="N6" s="6">
+        <f t="shared" si="1"/>
+        <v>0.3</v>
+      </c>
+      <c r="O6" s="5">
+        <f t="shared" si="2"/>
+        <v>11.799999999999999</v>
+      </c>
+      <c r="P6" s="7">
+        <v>8.9999999999999998E-4</v>
+      </c>
+      <c r="Q6" s="3">
+        <f t="shared" si="3"/>
+        <v>10.799999999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" ht="15" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B7">
         <v>401190</v>
       </c>
       <c r="C7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" t="s">
         <v>23</v>
-      </c>
-      <c r="D7" t="s">
-        <v>24</v>
       </c>
       <c r="E7">
         <v>600</v>
@@ -949,34 +1123,56 @@
       <c r="F7" s="3">
         <v>18000</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="3">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="H7">
         <v>200</v>
       </c>
-      <c r="H7">
+      <c r="I7">
         <v>80</v>
       </c>
-      <c r="I7">
+      <c r="J7">
         <v>200</v>
       </c>
-      <c r="J7" t="s">
+      <c r="K7" t="s">
         <v>6</v>
       </c>
-      <c r="K7">
+      <c r="L7">
         <v>100</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+      <c r="M7" s="5">
+        <v>24.5</v>
+      </c>
+      <c r="N7" s="6">
+        <f t="shared" si="1"/>
+        <v>7.5</v>
+      </c>
+      <c r="O7" s="5">
+        <f t="shared" si="2"/>
+        <v>283.75</v>
+      </c>
+      <c r="P7" s="7">
+        <v>1.1999999999999999E-3</v>
+      </c>
+      <c r="Q7" s="3">
+        <f t="shared" si="3"/>
+        <v>3.5999999999999997E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" ht="15" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B8">
         <v>870829</v>
       </c>
       <c r="C8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E8">
         <v>30</v>
@@ -984,34 +1180,56 @@
       <c r="F8" s="3">
         <v>30000</v>
       </c>
-      <c r="G8">
+      <c r="G8" s="3">
+        <f t="shared" si="0"/>
+        <v>1000</v>
+      </c>
+      <c r="H8">
         <v>5</v>
       </c>
-      <c r="H8">
+      <c r="I8">
         <v>35</v>
       </c>
-      <c r="I8">
+      <c r="J8">
         <v>5</v>
       </c>
-      <c r="J8" t="s">
+      <c r="K8" t="s">
         <v>5</v>
       </c>
-      <c r="K8">
+      <c r="L8">
         <v>3</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+      <c r="M8" s="5">
+        <v>22.8</v>
+      </c>
+      <c r="N8" s="6">
+        <f t="shared" si="1"/>
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="O8" s="5">
+        <f t="shared" si="2"/>
+        <v>22.542857142857141</v>
+      </c>
+      <c r="P8" s="7">
+        <v>6.9999999999999999E-4</v>
+      </c>
+      <c r="Q8" s="3">
+        <f t="shared" si="3"/>
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" ht="15" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B9">
         <v>870899</v>
       </c>
       <c r="C9" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" t="s">
         <v>28</v>
-      </c>
-      <c r="D9" t="s">
-        <v>29</v>
       </c>
       <c r="E9">
         <v>20</v>
@@ -1019,34 +1237,56 @@
       <c r="F9" s="3">
         <v>40000</v>
       </c>
-      <c r="G9">
+      <c r="G9" s="3">
+        <f t="shared" si="0"/>
+        <v>2000</v>
+      </c>
+      <c r="H9">
         <v>3</v>
       </c>
-      <c r="H9">
+      <c r="I9">
         <v>40</v>
       </c>
-      <c r="I9">
+      <c r="J9">
         <v>5</v>
       </c>
-      <c r="J9" t="s">
+      <c r="K9" t="s">
         <v>5</v>
       </c>
-      <c r="K9">
+      <c r="L9">
         <v>2</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+      <c r="M9" s="5">
+        <v>38.4</v>
+      </c>
+      <c r="N9" s="6">
+        <f t="shared" si="1"/>
+        <v>0.5</v>
+      </c>
+      <c r="O9" s="5">
+        <f t="shared" si="2"/>
+        <v>21.2</v>
+      </c>
+      <c r="P9" s="7">
+        <v>1E-3</v>
+      </c>
+      <c r="Q9" s="3">
+        <f t="shared" si="3"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" ht="15" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B10">
         <v>870880</v>
       </c>
       <c r="C10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E10">
         <v>240</v>
@@ -1054,34 +1294,56 @@
       <c r="F10" s="3">
         <v>19200</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="3">
+        <f t="shared" si="0"/>
+        <v>80</v>
+      </c>
+      <c r="H10">
         <v>60</v>
       </c>
-      <c r="H10">
+      <c r="I10">
         <v>90</v>
       </c>
-      <c r="I10">
+      <c r="J10">
         <v>120</v>
       </c>
-      <c r="J10" t="s">
+      <c r="K10" t="s">
         <v>6</v>
       </c>
-      <c r="K10">
+      <c r="L10">
         <v>60</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+      <c r="M10" s="5">
+        <v>17.600000000000001</v>
+      </c>
+      <c r="N10" s="6">
+        <f t="shared" si="1"/>
+        <v>2.6666666666666665</v>
+      </c>
+      <c r="O10" s="5">
+        <f t="shared" si="2"/>
+        <v>106.93333333333334</v>
+      </c>
+      <c r="P10" s="7">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="Q10" s="3">
+        <f t="shared" si="3"/>
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" ht="15" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B11">
         <v>401110</v>
       </c>
       <c r="C11" t="s">
+        <v>32</v>
+      </c>
+      <c r="D11" t="s">
         <v>33</v>
-      </c>
-      <c r="D11" t="s">
-        <v>34</v>
       </c>
       <c r="E11">
         <v>500</v>
@@ -1089,34 +1351,56 @@
       <c r="F11" s="3">
         <v>25000</v>
       </c>
-      <c r="G11">
+      <c r="G11" s="3">
+        <f t="shared" si="0"/>
+        <v>50</v>
+      </c>
+      <c r="H11">
         <v>150</v>
       </c>
-      <c r="H11">
+      <c r="I11">
         <v>75</v>
       </c>
-      <c r="I11">
+      <c r="J11">
         <v>250</v>
       </c>
-      <c r="J11" t="s">
+      <c r="K11" t="s">
         <v>6</v>
       </c>
-      <c r="K11">
+      <c r="L11">
         <v>100</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+      <c r="M11" s="5">
+        <v>21.6</v>
+      </c>
+      <c r="N11" s="6">
+        <f t="shared" si="1"/>
+        <v>6.666666666666667</v>
+      </c>
+      <c r="O11" s="5">
+        <f t="shared" si="2"/>
+        <v>244.00000000000003</v>
+      </c>
+      <c r="P11" s="7">
+        <v>1.2999999999999999E-3</v>
+      </c>
+      <c r="Q11" s="3">
+        <f t="shared" si="3"/>
+        <v>6.5000000000000002E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" ht="15" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B12">
         <v>401110</v>
       </c>
       <c r="C12" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E12">
         <v>80</v>
@@ -1124,25 +1408,47 @@
       <c r="F12" s="3">
         <v>64000</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="3">
+        <f t="shared" si="0"/>
+        <v>800</v>
+      </c>
+      <c r="H12">
         <v>20</v>
       </c>
-      <c r="H12">
+      <c r="I12">
         <v>60</v>
       </c>
-      <c r="I12">
+      <c r="J12">
         <v>10</v>
       </c>
-      <c r="J12" t="s">
+      <c r="K12" t="s">
         <v>5</v>
       </c>
-      <c r="K12">
+      <c r="L12">
         <v>5</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+      <c r="M12" s="5">
+        <v>43</v>
+      </c>
+      <c r="N12" s="6">
+        <f t="shared" si="1"/>
+        <v>1.3333333333333333</v>
+      </c>
+      <c r="O12" s="5">
+        <f t="shared" si="2"/>
+        <v>62.333333333333329</v>
+      </c>
+      <c r="P12" s="7">
+        <v>8.0000000000000004E-4</v>
+      </c>
+      <c r="Q12" s="3">
+        <f t="shared" si="3"/>
+        <v>0.64</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" ht="15" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B13">
         <v>840999</v>
@@ -1151,7 +1457,7 @@
         <v>7</v>
       </c>
       <c r="D13" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E13">
         <v>35</v>
@@ -1159,25 +1465,47 @@
       <c r="F13" s="3">
         <v>17500</v>
       </c>
-      <c r="G13">
+      <c r="G13" s="3">
+        <f t="shared" si="0"/>
+        <v>500</v>
+      </c>
+      <c r="H13">
         <v>10</v>
       </c>
-      <c r="H13">
+      <c r="I13">
         <v>40</v>
       </c>
-      <c r="I13">
+      <c r="J13">
         <v>10</v>
       </c>
-      <c r="J13" t="s">
+      <c r="K13" t="s">
         <v>5</v>
       </c>
-      <c r="K13">
+      <c r="L13">
         <v>4</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+      <c r="M13" s="5">
+        <v>16.8</v>
+      </c>
+      <c r="N13" s="6">
+        <f t="shared" si="1"/>
+        <v>0.875</v>
+      </c>
+      <c r="O13" s="5">
+        <f t="shared" si="2"/>
+        <v>18.700000000000003</v>
+      </c>
+      <c r="P13" s="7">
+        <v>1.1000000000000001E-3</v>
+      </c>
+      <c r="Q13" s="3">
+        <f t="shared" si="3"/>
+        <v>0.55000000000000004</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" ht="15" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B14">
         <v>850710</v>
@@ -1186,7 +1514,7 @@
         <v>7</v>
       </c>
       <c r="D14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E14">
         <v>28</v>
@@ -1194,25 +1522,47 @@
       <c r="F14" s="3">
         <v>16800</v>
       </c>
-      <c r="G14">
+      <c r="G14" s="3">
+        <f t="shared" si="0"/>
+        <v>600</v>
+      </c>
+      <c r="H14">
         <v>6</v>
       </c>
-      <c r="H14">
+      <c r="I14">
         <v>38</v>
       </c>
-      <c r="I14">
+      <c r="J14">
         <v>8</v>
       </c>
-      <c r="J14" t="s">
+      <c r="K14" t="s">
         <v>5</v>
       </c>
-      <c r="K14">
+      <c r="L14">
         <v>3</v>
       </c>
-    </row>
-    <row r="15" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+      <c r="M14" s="5">
+        <v>23.4</v>
+      </c>
+      <c r="N14" s="6">
+        <f t="shared" si="1"/>
+        <v>0.73684210526315785</v>
+      </c>
+      <c r="O14" s="5">
+        <f t="shared" si="2"/>
+        <v>20.242105263157892</v>
+      </c>
+      <c r="P14" s="7">
+        <v>5.9999999999999995E-4</v>
+      </c>
+      <c r="Q14" s="3">
+        <f t="shared" si="3"/>
+        <v>0.36</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" ht="15" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B15">
         <v>851220</v>
@@ -1221,7 +1571,7 @@
         <v>7</v>
       </c>
       <c r="D15" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E15">
         <v>15</v>
@@ -1229,34 +1579,56 @@
       <c r="F15" s="3">
         <v>90000</v>
       </c>
-      <c r="G15">
+      <c r="G15" s="3">
+        <f t="shared" si="0"/>
+        <v>6000</v>
+      </c>
+      <c r="H15">
         <v>4</v>
       </c>
-      <c r="H15">
+      <c r="I15">
         <v>30</v>
       </c>
-      <c r="I15">
+      <c r="J15">
         <v>2</v>
       </c>
-      <c r="J15" t="s">
+      <c r="K15" t="s">
         <v>5</v>
       </c>
-      <c r="K15">
+      <c r="L15">
         <v>1</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+      <c r="M15" s="5">
+        <v>27.6</v>
+      </c>
+      <c r="N15" s="6">
+        <f t="shared" si="1"/>
+        <v>0.5</v>
+      </c>
+      <c r="O15" s="5">
+        <f t="shared" si="2"/>
+        <v>14.8</v>
+      </c>
+      <c r="P15" s="7">
+        <v>1.4E-3</v>
+      </c>
+      <c r="Q15" s="3">
+        <f t="shared" si="3"/>
+        <v>8.4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" ht="15" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B16">
         <v>870829</v>
       </c>
       <c r="C16" t="s">
+        <v>43</v>
+      </c>
+      <c r="D16" t="s">
         <v>44</v>
-      </c>
-      <c r="D16" t="s">
-        <v>45</v>
       </c>
       <c r="E16">
         <v>55</v>
@@ -1264,34 +1636,56 @@
       <c r="F16" s="3">
         <v>22000</v>
       </c>
-      <c r="G16">
+      <c r="G16" s="3">
+        <f t="shared" si="0"/>
+        <v>400</v>
+      </c>
+      <c r="H16">
         <v>12</v>
       </c>
-      <c r="H16">
+      <c r="I16">
         <v>50</v>
       </c>
-      <c r="I16">
+      <c r="J16">
         <v>10</v>
       </c>
-      <c r="J16" t="s">
+      <c r="K16" t="s">
         <v>5</v>
       </c>
-      <c r="K16">
+      <c r="L16">
         <v>5</v>
       </c>
-    </row>
-    <row r="17" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+      <c r="M16" s="5">
+        <v>20.6</v>
+      </c>
+      <c r="N16" s="6">
+        <f t="shared" si="1"/>
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="O16" s="5">
+        <f t="shared" si="2"/>
+        <v>27.660000000000004</v>
+      </c>
+      <c r="P16" s="7">
+        <v>8.9999999999999998E-4</v>
+      </c>
+      <c r="Q16" s="3">
+        <f t="shared" si="3"/>
+        <v>0.36</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" ht="15" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B17">
         <v>870810</v>
       </c>
       <c r="C17" t="s">
+        <v>46</v>
+      </c>
+      <c r="D17" t="s">
         <v>47</v>
-      </c>
-      <c r="D17" t="s">
-        <v>48</v>
       </c>
       <c r="E17">
         <v>40</v>
@@ -1299,34 +1693,56 @@
       <c r="F17" s="3">
         <v>32000</v>
       </c>
-      <c r="G17">
+      <c r="G17" s="3">
+        <f t="shared" si="0"/>
+        <v>800</v>
+      </c>
+      <c r="H17">
         <v>8</v>
       </c>
-      <c r="H17">
+      <c r="I17">
         <v>65</v>
       </c>
-      <c r="I17">
+      <c r="J17">
         <v>5</v>
       </c>
-      <c r="J17" t="s">
+      <c r="K17" t="s">
         <v>6</v>
       </c>
-      <c r="K17">
+      <c r="L17">
         <v>3</v>
       </c>
-    </row>
-    <row r="18" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+      <c r="M17" s="5">
+        <v>32.9</v>
+      </c>
+      <c r="N17" s="6">
+        <f t="shared" si="1"/>
+        <v>0.61538461538461542</v>
+      </c>
+      <c r="O17" s="5">
+        <f t="shared" si="2"/>
+        <v>23.246153846153845</v>
+      </c>
+      <c r="P17" s="7">
+        <v>1.1999999999999999E-3</v>
+      </c>
+      <c r="Q17" s="3">
+        <f t="shared" si="3"/>
+        <v>0.96</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" ht="15" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B18">
         <v>870899</v>
       </c>
       <c r="C18" t="s">
+        <v>49</v>
+      </c>
+      <c r="D18" t="s">
         <v>50</v>
-      </c>
-      <c r="D18" t="s">
-        <v>51</v>
       </c>
       <c r="E18">
         <v>18</v>
@@ -1334,34 +1750,56 @@
       <c r="F18" s="3">
         <v>12600</v>
       </c>
-      <c r="G18">
+      <c r="G18" s="3">
+        <f t="shared" si="0"/>
+        <v>700</v>
+      </c>
+      <c r="H18">
         <v>5</v>
       </c>
-      <c r="H18">
+      <c r="I18">
         <v>45</v>
       </c>
-      <c r="I18">
+      <c r="J18">
         <v>5</v>
       </c>
-      <c r="J18" t="s">
+      <c r="K18" t="s">
         <v>5</v>
       </c>
-      <c r="K18">
+      <c r="L18">
         <v>2</v>
       </c>
-    </row>
-    <row r="19" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+      <c r="M18" s="5">
+        <v>25.1</v>
+      </c>
+      <c r="N18" s="6">
+        <f t="shared" si="1"/>
+        <v>0.4</v>
+      </c>
+      <c r="O18" s="5">
+        <f t="shared" si="2"/>
+        <v>12.040000000000001</v>
+      </c>
+      <c r="P18" s="7">
+        <v>6.9999999999999999E-4</v>
+      </c>
+      <c r="Q18" s="3">
+        <f t="shared" si="3"/>
+        <v>0.49</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" ht="15" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B19">
         <v>870870</v>
       </c>
       <c r="C19" t="s">
+        <v>52</v>
+      </c>
+      <c r="D19" t="s">
         <v>53</v>
-      </c>
-      <c r="D19" t="s">
-        <v>54</v>
       </c>
       <c r="E19">
         <v>2000</v>
@@ -1369,34 +1807,56 @@
       <c r="F19" s="3">
         <v>4000</v>
       </c>
-      <c r="G19">
+      <c r="G19" s="3">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="H19">
         <v>500</v>
       </c>
-      <c r="H19">
+      <c r="I19">
         <v>120</v>
       </c>
-      <c r="I19">
+      <c r="J19">
         <v>1000</v>
       </c>
-      <c r="J19" t="s">
+      <c r="K19" t="s">
         <v>6</v>
       </c>
-      <c r="K19">
+      <c r="L19">
         <v>300</v>
       </c>
-    </row>
-    <row r="20" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+      <c r="M19" s="5">
+        <v>15.15</v>
+      </c>
+      <c r="N19" s="6">
+        <f t="shared" si="1"/>
+        <v>16.666666666666668</v>
+      </c>
+      <c r="O19" s="5">
+        <f t="shared" si="2"/>
+        <v>552.5</v>
+      </c>
+      <c r="P19" s="7">
+        <v>1E-3</v>
+      </c>
+      <c r="Q19" s="3">
+        <f t="shared" si="3"/>
+        <v>2E-3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" ht="15" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B20">
         <v>870880</v>
       </c>
       <c r="C20" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D20" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E20">
         <v>180</v>
@@ -1404,34 +1864,56 @@
       <c r="F20" s="3">
         <v>32400</v>
       </c>
-      <c r="G20">
+      <c r="G20" s="3">
+        <f t="shared" si="0"/>
+        <v>180</v>
+      </c>
+      <c r="H20">
         <v>50</v>
       </c>
-      <c r="H20">
+      <c r="I20">
         <v>55</v>
       </c>
-      <c r="I20">
+      <c r="J20">
         <v>100</v>
       </c>
-      <c r="J20" t="s">
+      <c r="K20" t="s">
         <v>6</v>
       </c>
-      <c r="K20">
+      <c r="L20">
         <v>40</v>
       </c>
-    </row>
-    <row r="21" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+      <c r="M20" s="5">
+        <v>34.5</v>
+      </c>
+      <c r="N20" s="6">
+        <f t="shared" si="1"/>
+        <v>3.2727272727272729</v>
+      </c>
+      <c r="O20" s="5">
+        <f t="shared" si="2"/>
+        <v>152.90909090909093</v>
+      </c>
+      <c r="P20" s="7">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="Q20" s="3">
+        <f t="shared" si="3"/>
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" ht="15" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B21">
         <v>870829</v>
       </c>
       <c r="C21" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D21" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E21">
         <v>360</v>
@@ -1439,34 +1921,56 @@
       <c r="F21" s="3">
         <v>28800</v>
       </c>
-      <c r="G21">
+      <c r="G21" s="3">
+        <f t="shared" si="0"/>
         <v>80</v>
       </c>
       <c r="H21">
+        <v>80</v>
+      </c>
+      <c r="I21">
         <v>95</v>
       </c>
-      <c r="I21">
+      <c r="J21">
         <v>200</v>
       </c>
-      <c r="J21" t="s">
+      <c r="K21" t="s">
         <v>6</v>
       </c>
-      <c r="K21">
+      <c r="L21">
         <v>80</v>
       </c>
-    </row>
-    <row r="22" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+      <c r="M21" s="5">
+        <v>27</v>
+      </c>
+      <c r="N21" s="6">
+        <f t="shared" si="1"/>
+        <v>3.7894736842105261</v>
+      </c>
+      <c r="O21" s="5">
+        <f t="shared" si="2"/>
+        <v>182.31578947368422</v>
+      </c>
+      <c r="P21" s="7">
+        <v>1.2999999999999999E-3</v>
+      </c>
+      <c r="Q21" s="3">
+        <f t="shared" si="3"/>
+        <v>0.104</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" ht="15" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B22">
         <v>870840</v>
       </c>
       <c r="C22" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D22" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E22">
         <v>150</v>
@@ -1474,34 +1978,56 @@
       <c r="F22" s="3">
         <v>4500</v>
       </c>
-      <c r="G22">
+      <c r="G22" s="3">
+        <f t="shared" si="0"/>
         <v>30</v>
       </c>
       <c r="H22">
+        <v>30</v>
+      </c>
+      <c r="I22">
         <v>70</v>
       </c>
-      <c r="I22">
+      <c r="J22">
         <v>150</v>
       </c>
-      <c r="J22" t="s">
+      <c r="K22" t="s">
         <v>6</v>
       </c>
-      <c r="K22">
+      <c r="L22">
         <v>50</v>
       </c>
-    </row>
-    <row r="23" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+      <c r="M22" s="5">
+        <v>22.799999999999997</v>
+      </c>
+      <c r="N22" s="6">
+        <f t="shared" si="1"/>
+        <v>2.1428571428571428</v>
+      </c>
+      <c r="O22" s="5">
+        <f t="shared" si="2"/>
+        <v>98.857142857142847</v>
+      </c>
+      <c r="P22" s="7">
+        <v>8.0000000000000004E-4</v>
+      </c>
+      <c r="Q22" s="3">
+        <f t="shared" si="3"/>
+        <v>2.4E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" ht="15" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B23">
         <v>840991</v>
       </c>
       <c r="C23" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E23">
         <v>90</v>
@@ -1509,25 +2035,47 @@
       <c r="F23" s="3">
         <v>27000</v>
       </c>
-      <c r="G23">
+      <c r="G23" s="3">
+        <f t="shared" si="0"/>
+        <v>300</v>
+      </c>
+      <c r="H23">
         <v>25</v>
       </c>
-      <c r="H23">
+      <c r="I23">
         <v>45</v>
       </c>
-      <c r="I23">
+      <c r="J23">
         <v>50</v>
       </c>
-      <c r="J23" t="s">
+      <c r="K23" t="s">
         <v>5</v>
       </c>
-      <c r="K23">
+      <c r="L23">
         <v>20</v>
       </c>
-    </row>
-    <row r="24" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+      <c r="M23" s="5">
+        <v>18.399999999999999</v>
+      </c>
+      <c r="N23" s="6">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="O23" s="5">
+        <f t="shared" si="2"/>
+        <v>56.8</v>
+      </c>
+      <c r="P23" s="7">
+        <v>1.1000000000000001E-3</v>
+      </c>
+      <c r="Q23" s="3">
+        <f t="shared" si="3"/>
+        <v>0.33</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" ht="15" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B24">
         <v>901829</v>
@@ -1536,7 +2084,7 @@
         <v>7</v>
       </c>
       <c r="D24" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E24">
         <v>480</v>
@@ -1544,34 +2092,56 @@
       <c r="F24" s="3">
         <v>9600</v>
       </c>
-      <c r="G24">
+      <c r="G24" s="3">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="H24">
         <v>120</v>
       </c>
-      <c r="H24">
+      <c r="I24">
         <v>100</v>
       </c>
-      <c r="I24">
+      <c r="J24">
         <v>300</v>
       </c>
-      <c r="J24" t="s">
+      <c r="K24" t="s">
         <v>6</v>
       </c>
-      <c r="K24">
+      <c r="L24">
         <v>150</v>
       </c>
-    </row>
-    <row r="25" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+      <c r="M24" s="5">
+        <v>18.5</v>
+      </c>
+      <c r="N24" s="6">
+        <f t="shared" si="1"/>
+        <v>4.8</v>
+      </c>
+      <c r="O24" s="5">
+        <f t="shared" si="2"/>
+        <v>238.8</v>
+      </c>
+      <c r="P24" s="7">
+        <v>5.9999999999999995E-4</v>
+      </c>
+      <c r="Q24" s="3">
+        <f t="shared" si="3"/>
+        <v>1.1999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" ht="15" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B25">
         <v>870899</v>
       </c>
       <c r="C25" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D25" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E25">
         <v>260</v>
@@ -1579,34 +2149,56 @@
       <c r="F25" s="3">
         <v>52000</v>
       </c>
-      <c r="G25">
+      <c r="G25" s="3">
+        <f t="shared" si="0"/>
+        <v>200</v>
+      </c>
+      <c r="H25">
         <v>60</v>
       </c>
-      <c r="H25">
+      <c r="I25">
         <v>85</v>
       </c>
-      <c r="I25">
+      <c r="J25">
         <v>200</v>
       </c>
-      <c r="J25" t="s">
+      <c r="K25" t="s">
         <v>6</v>
       </c>
-      <c r="K25">
+      <c r="L25">
         <v>100</v>
       </c>
-    </row>
-    <row r="26" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+      <c r="M25" s="5">
+        <v>26</v>
+      </c>
+      <c r="N25" s="6">
+        <f t="shared" si="1"/>
+        <v>3.0588235294117645</v>
+      </c>
+      <c r="O25" s="5">
+        <f t="shared" si="2"/>
+        <v>179.52941176470588</v>
+      </c>
+      <c r="P25" s="7">
+        <v>1.4E-3</v>
+      </c>
+      <c r="Q25" s="3">
+        <f t="shared" si="3"/>
+        <v>0.27999999999999997</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" ht="15" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B26">
         <v>870829</v>
       </c>
       <c r="C26" t="s">
+        <v>67</v>
+      </c>
+      <c r="D26" t="s">
         <v>68</v>
-      </c>
-      <c r="D26" t="s">
-        <v>69</v>
       </c>
       <c r="E26">
         <v>38</v>
@@ -1614,34 +2206,56 @@
       <c r="F26" s="3">
         <v>7600</v>
       </c>
-      <c r="G26">
+      <c r="G26" s="3">
+        <f t="shared" si="0"/>
+        <v>200</v>
+      </c>
+      <c r="H26">
         <v>10</v>
       </c>
-      <c r="H26">
+      <c r="I26">
         <v>50</v>
       </c>
-      <c r="I26">
+      <c r="J26">
         <v>20</v>
       </c>
-      <c r="J26" t="s">
+      <c r="K26" t="s">
         <v>5</v>
       </c>
-      <c r="K26">
+      <c r="L26">
         <v>8</v>
       </c>
-    </row>
-    <row r="27" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+      <c r="M26" s="5">
+        <v>23.799999999999997</v>
+      </c>
+      <c r="N26" s="6">
+        <f t="shared" si="1"/>
+        <v>0.76</v>
+      </c>
+      <c r="O26" s="5">
+        <f t="shared" si="2"/>
+        <v>26.087999999999997</v>
+      </c>
+      <c r="P26" s="7">
+        <v>8.9999999999999998E-4</v>
+      </c>
+      <c r="Q26" s="3">
+        <f t="shared" si="3"/>
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" ht="15" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B27">
         <v>841459</v>
       </c>
       <c r="C27" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D27" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E27">
         <v>32</v>
@@ -1649,34 +2263,56 @@
       <c r="F27" s="3">
         <v>12800</v>
       </c>
-      <c r="G27">
+      <c r="G27" s="3">
+        <f t="shared" si="0"/>
+        <v>400</v>
+      </c>
+      <c r="H27">
         <v>6</v>
       </c>
-      <c r="H27">
+      <c r="I27">
         <v>48</v>
       </c>
-      <c r="I27">
+      <c r="J27">
         <v>10</v>
       </c>
-      <c r="J27" t="s">
+      <c r="K27" t="s">
         <v>5</v>
       </c>
-      <c r="K27">
+      <c r="L27">
         <v>5</v>
       </c>
-    </row>
-    <row r="28" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+      <c r="M27" s="5">
+        <v>29.8</v>
+      </c>
+      <c r="N27" s="6">
+        <f t="shared" si="1"/>
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="O27" s="5">
+        <f t="shared" si="2"/>
+        <v>24.866666666666667</v>
+      </c>
+      <c r="P27" s="7">
+        <v>1.1999999999999999E-3</v>
+      </c>
+      <c r="Q27" s="3">
+        <f t="shared" si="3"/>
+        <v>0.48</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" ht="15" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B28">
         <v>401190</v>
       </c>
       <c r="C28" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D28" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E28">
         <v>1200</v>
@@ -1684,34 +2320,56 @@
       <c r="F28" s="3">
         <v>180000</v>
       </c>
-      <c r="G28">
+      <c r="G28" s="3">
+        <f t="shared" si="0"/>
+        <v>150</v>
+      </c>
+      <c r="H28">
         <v>400</v>
       </c>
-      <c r="H28">
+      <c r="I28">
         <v>30</v>
       </c>
-      <c r="I28">
+      <c r="J28">
         <v>2000</v>
       </c>
-      <c r="J28" t="s">
+      <c r="K28" t="s">
         <v>6</v>
       </c>
-      <c r="K28">
+      <c r="L28">
         <v>600</v>
       </c>
-    </row>
-    <row r="29" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+      <c r="M28" s="5">
+        <v>17.5</v>
+      </c>
+      <c r="N28" s="6">
+        <f t="shared" si="1"/>
+        <v>40</v>
+      </c>
+      <c r="O28" s="5">
+        <f t="shared" si="2"/>
+        <v>1300</v>
+      </c>
+      <c r="P28" s="7">
+        <v>6.9999999999999999E-4</v>
+      </c>
+      <c r="Q28" s="3">
+        <f t="shared" si="3"/>
+        <v>0.105</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" ht="15" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B29">
         <v>870899</v>
       </c>
       <c r="C29" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D29" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E29">
         <v>240</v>
@@ -1719,34 +2377,56 @@
       <c r="F29" s="3">
         <v>9600</v>
       </c>
-      <c r="G29">
+      <c r="G29" s="3">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+      <c r="H29">
         <v>50</v>
       </c>
-      <c r="H29">
+      <c r="I29">
         <v>110</v>
       </c>
-      <c r="I29">
+      <c r="J29">
         <v>300</v>
       </c>
-      <c r="J29" t="s">
+      <c r="K29" t="s">
         <v>6</v>
       </c>
-      <c r="K29">
+      <c r="L29">
         <v>100</v>
       </c>
-    </row>
-    <row r="30" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+      <c r="M29" s="5">
+        <v>25.2</v>
+      </c>
+      <c r="N29" s="6">
+        <f t="shared" si="1"/>
+        <v>2.1818181818181817</v>
+      </c>
+      <c r="O29" s="5">
+        <f t="shared" si="2"/>
+        <v>154.98181818181817</v>
+      </c>
+      <c r="P29" s="7">
+        <v>1E-3</v>
+      </c>
+      <c r="Q29" s="3">
+        <f t="shared" si="3"/>
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17" ht="15" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B30">
         <v>870899</v>
       </c>
       <c r="C30" t="s">
+        <v>76</v>
+      </c>
+      <c r="D30" t="s">
         <v>77</v>
-      </c>
-      <c r="D30" t="s">
-        <v>78</v>
       </c>
       <c r="E30">
         <v>1500</v>
@@ -1754,25 +2434,47 @@
       <c r="F30" s="3">
         <v>22500</v>
       </c>
-      <c r="G30">
+      <c r="G30" s="3">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="H30">
         <v>400</v>
       </c>
-      <c r="H30">
+      <c r="I30">
         <v>150</v>
       </c>
-      <c r="I30">
+      <c r="J30">
         <v>2000</v>
       </c>
-      <c r="J30" t="s">
+      <c r="K30" t="s">
         <v>6</v>
       </c>
-      <c r="K30">
+      <c r="L30">
         <v>500</v>
       </c>
-    </row>
-    <row r="31" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+      <c r="M30" s="5">
+        <v>29.200000000000003</v>
+      </c>
+      <c r="N30" s="6">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="O30" s="5">
+        <f t="shared" si="2"/>
+        <v>792</v>
+      </c>
+      <c r="P30" s="7">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="Q30" s="3">
+        <f t="shared" si="3"/>
+        <v>7.4999999999999997E-3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17" ht="15" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B31">
         <v>870829</v>
@@ -1781,7 +2483,7 @@
         <v>7</v>
       </c>
       <c r="D31" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E31">
         <v>420</v>
@@ -1789,28 +2491,70 @@
       <c r="F31" s="3">
         <v>6300</v>
       </c>
-      <c r="G31">
+      <c r="G31" s="3">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="H31">
         <v>80</v>
       </c>
-      <c r="H31">
+      <c r="I31">
         <v>95</v>
       </c>
-      <c r="I31">
+      <c r="J31">
         <v>200</v>
       </c>
-      <c r="J31" t="s">
+      <c r="K31" t="s">
         <v>6</v>
       </c>
-      <c r="K31">
+      <c r="L31">
         <v>100</v>
+      </c>
+      <c r="M31" s="5">
+        <v>19.8</v>
+      </c>
+      <c r="N31" s="6">
+        <f t="shared" si="1"/>
+        <v>4.4210526315789478</v>
+      </c>
+      <c r="O31" s="5">
+        <f t="shared" si="2"/>
+        <v>187.53684210526319</v>
+      </c>
+      <c r="P31" s="7">
+        <v>1.2999999999999999E-3</v>
+      </c>
+      <c r="Q31" s="3">
+        <f t="shared" si="3"/>
+        <v>1.95E-2</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="942691e6-3dd6-4136-b9de-ea5482bfa647">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101007A0A104EFF5C024AA79AD78CB44176CF" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="20cf8a6f49ef8bb54dd1547e2829c48f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="942691e6-3dd6-4136-b9de-ea5482bfa647" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1183328a354284f1910a6057b013db4c" ns2:_="">
     <xsd:import namespace="942691e6-3dd6-4136-b9de-ea5482bfa647"/>
@@ -1994,39 +2738,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="942691e6-3dd6-4136-b9de-ea5482bfa647">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8268C67-B164-4636-9D95-8793FBE5E6F5}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AE23CFE5-4C48-4888-9500-BC95E1CC93A1}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="942691e6-3dd6-4136-b9de-ea5482bfa647"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2048,9 +2763,19 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AE23CFE5-4C48-4888-9500-BC95E1CC93A1}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8268C67-B164-4636-9D95-8793FBE5E6F5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="942691e6-3dd6-4136-b9de-ea5482bfa647"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>